<commit_message>
chore: update crypto volume snapshot
</commit_message>
<xml_diff>
--- a/crypto_volume.xlsx
+++ b/crypto_volume.xlsx
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>593659004.78</v>
+        <v>231381100.46</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -481,7 +481,7 @@
         </is>
       </c>
       <c r="F2" s="1" t="n">
-        <v>509018831.46</v>
+        <v>228487736.4</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -489,7 +489,7 @@
         </is>
       </c>
       <c r="I2" s="1" t="n">
-        <v>6172839.619255594</v>
+        <v>3754624.229601813</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -497,7 +497,7 @@
         </is>
       </c>
       <c r="L2" s="1" t="n">
-        <v>8172085.73</v>
+        <v>1608892.46</v>
       </c>
     </row>
     <row r="3">
@@ -510,7 +510,7 @@
         </is>
       </c>
       <c r="C3" s="1" t="n">
-        <v>251396735.47</v>
+        <v>40970669.84</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -518,23 +518,23 @@
         </is>
       </c>
       <c r="F3" s="1" t="n">
-        <v>60735421.09402</v>
+        <v>53781951.59154</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>BTC_THB</t>
+          <t>ETH_THB</t>
         </is>
       </c>
       <c r="I3" s="1" t="n">
-        <v>4940024.275329733</v>
+        <v>326404.9117164645</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>ETHTHB</t>
+          <t>UNITHB</t>
         </is>
       </c>
       <c r="L3" s="1" t="n">
-        <v>3797181.24</v>
+        <v>606523.67</v>
       </c>
     </row>
     <row r="4">
@@ -547,31 +547,31 @@
         </is>
       </c>
       <c r="C4" s="1" t="n">
-        <v>229420778.12</v>
+        <v>31722471.51</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>VELOTHB</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="n">
+        <v>1837211.5926</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>XRP_THB</t>
+        </is>
+      </c>
+      <c r="I4" s="1" t="n">
+        <v>210650.4004093856</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
           <t>ETHTHB</t>
         </is>
       </c>
-      <c r="F4" s="1" t="n">
-        <v>19520106.3651</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>ETH_THB</t>
-        </is>
-      </c>
-      <c r="I4" s="1" t="n">
-        <v>4891661.252085375</v>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>XRPTHB</t>
-        </is>
-      </c>
       <c r="L4" s="1" t="n">
-        <v>2599120.01</v>
+        <v>263159.39</v>
       </c>
     </row>
     <row r="5">
@@ -580,35 +580,35 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>THB_NEAR</t>
+          <t>THB_XRP</t>
         </is>
       </c>
       <c r="C5" s="1" t="n">
-        <v>68941260.34</v>
+        <v>15235084.53</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>XRPTHB</t>
+          <t>ETHTHB</t>
         </is>
       </c>
       <c r="F5" s="1" t="n">
-        <v>3545289.5395</v>
+        <v>1553285.7466</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>XRP_THB</t>
+          <t>BTC_THB</t>
         </is>
       </c>
       <c r="I5" s="1" t="n">
-        <v>352505.4884084313</v>
+        <v>159808.6975110888</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>USDTTHB</t>
+          <t>NEARTHB</t>
         </is>
       </c>
       <c r="L5" s="1" t="n">
-        <v>1231200.46</v>
+        <v>247852.44</v>
       </c>
     </row>
     <row r="6">
@@ -617,35 +617,35 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>THB_XRP</t>
+          <t>THB_NEAR</t>
         </is>
       </c>
       <c r="C6" s="1" t="n">
-        <v>60364643.44</v>
+        <v>11000703.55</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>VELOTHB</t>
+          <t>XRPTHB</t>
         </is>
       </c>
       <c r="F6" s="1" t="n">
-        <v>2413397.7377</v>
+        <v>728928.2594</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>XAUT_THB</t>
+          <t>SOL_THB</t>
         </is>
       </c>
       <c r="I6" s="1" t="n">
-        <v>169942.899</v>
+        <v>92454.4904311326</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>SOLTHB</t>
+          <t>SUSHITHB</t>
         </is>
       </c>
       <c r="L6" s="1" t="n">
-        <v>797466.3199999999</v>
+        <v>109182.29</v>
       </c>
     </row>
     <row r="7"/>
@@ -662,7 +662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BXW18"/>
+  <dimension ref="A1:BXW19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22732,6 +22732,1083 @@
         <v>103.08</v>
       </c>
       <c r="PV18" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>13</v>
+      </c>
+      <c r="B19" s="1" t="n">
+        <v>231381100.46</v>
+      </c>
+      <c r="C19" s="1" t="n">
+        <v>40970669.84</v>
+      </c>
+      <c r="D19" s="1">
+        <f>AVERAGE(C13:C19)</f>
+        <v/>
+      </c>
+      <c r="E19" s="1" t="n">
+        <v>31722471.51</v>
+      </c>
+      <c r="F19" s="1" t="n">
+        <v>15235084.53</v>
+      </c>
+      <c r="G19" s="1" t="n">
+        <v>6392247.84</v>
+      </c>
+      <c r="H19" s="1" t="n">
+        <v>7167880.36</v>
+      </c>
+      <c r="I19" s="1" t="n">
+        <v>2711934.45</v>
+      </c>
+      <c r="J19" s="1" t="n">
+        <v>3821234.52</v>
+      </c>
+      <c r="K19" s="1" t="n">
+        <v>1248897.43</v>
+      </c>
+      <c r="L19" s="1" t="n">
+        <v>3997644.28</v>
+      </c>
+      <c r="M19" s="1" t="n">
+        <v>883414.26</v>
+      </c>
+      <c r="N19" s="1" t="n">
+        <v>11000703.55</v>
+      </c>
+      <c r="O19" s="1" t="n">
+        <v>2369188.08</v>
+      </c>
+      <c r="P19" s="1" t="n">
+        <v>20920.72</v>
+      </c>
+      <c r="Q19" s="1" t="n">
+        <v>1263509.69</v>
+      </c>
+      <c r="R19" s="1" t="n">
+        <v>8696156.35</v>
+      </c>
+      <c r="S19" s="1" t="n">
+        <v>2055600.9</v>
+      </c>
+      <c r="T19" s="1" t="n">
+        <v>2025864.95</v>
+      </c>
+      <c r="U19" s="1" t="n">
+        <v>2436786.2</v>
+      </c>
+      <c r="V19" s="1" t="n">
+        <v>75566.32000000001</v>
+      </c>
+      <c r="W19" s="1" t="n">
+        <v>2099736.55</v>
+      </c>
+      <c r="Y19" s="1" t="n">
+        <v>18016.08</v>
+      </c>
+      <c r="Z19" s="1" t="n">
+        <v>252702.71</v>
+      </c>
+      <c r="AA19" s="1" t="n">
+        <v>833398.11</v>
+      </c>
+      <c r="AB19" s="1" t="n">
+        <v>2467499.26</v>
+      </c>
+      <c r="AC19" s="1" t="n">
+        <v>2839180.94</v>
+      </c>
+      <c r="AD19" s="1" t="n">
+        <v>993096.67</v>
+      </c>
+      <c r="AE19" s="1" t="n">
+        <v>414451.06</v>
+      </c>
+      <c r="AF19" s="1" t="n">
+        <v>261676.08</v>
+      </c>
+      <c r="AG19" s="1" t="n">
+        <v>1941811.36</v>
+      </c>
+      <c r="AH19" s="1" t="n">
+        <v>104448.39</v>
+      </c>
+      <c r="AI19" s="1" t="n">
+        <v>3281294.82</v>
+      </c>
+      <c r="AJ19" s="1" t="n">
+        <v>3659731.02</v>
+      </c>
+      <c r="AK19" s="1" t="n">
+        <v>1048616.56</v>
+      </c>
+      <c r="AL19" s="1" t="n">
+        <v>1069444.09</v>
+      </c>
+      <c r="AN19" s="1" t="n">
+        <v>763488.12</v>
+      </c>
+      <c r="AO19" s="1" t="n">
+        <v>687195.71</v>
+      </c>
+      <c r="AP19" s="1" t="n">
+        <v>343811.68</v>
+      </c>
+      <c r="AQ19" s="1" t="n">
+        <v>587051.95</v>
+      </c>
+      <c r="AR19" s="1" t="n">
+        <v>415559.49</v>
+      </c>
+      <c r="AS19" s="1" t="n">
+        <v>142604.81</v>
+      </c>
+      <c r="AT19" s="1" t="n">
+        <v>2591695.44</v>
+      </c>
+      <c r="AU19" s="1" t="n">
+        <v>363892.12</v>
+      </c>
+      <c r="AV19" s="1" t="n">
+        <v>351890.34</v>
+      </c>
+      <c r="AW19" s="1" t="n">
+        <v>2162788.09</v>
+      </c>
+      <c r="AX19" s="1" t="n">
+        <v>200142.07</v>
+      </c>
+      <c r="AY19" s="1" t="n">
+        <v>51303.82</v>
+      </c>
+      <c r="AZ19" s="1" t="n">
+        <v>118665.71</v>
+      </c>
+      <c r="BA19" s="1" t="n">
+        <v>4189.42</v>
+      </c>
+      <c r="BB19" s="1" t="n">
+        <v>592716.27</v>
+      </c>
+      <c r="BC19" s="1" t="n">
+        <v>2193244.83</v>
+      </c>
+      <c r="BD19" s="1" t="n">
+        <v>93640.85000000001</v>
+      </c>
+      <c r="BE19" s="1" t="n">
+        <v>464226.46</v>
+      </c>
+      <c r="BF19" s="1" t="n">
+        <v>372895.88</v>
+      </c>
+      <c r="BG19" s="1" t="n">
+        <v>55745.18</v>
+      </c>
+      <c r="BI19" s="1" t="n">
+        <v>695.02</v>
+      </c>
+      <c r="BJ19" s="1" t="n">
+        <v>6651.21</v>
+      </c>
+      <c r="BK19" s="1" t="n">
+        <v>501539.08</v>
+      </c>
+      <c r="BL19" s="1" t="n">
+        <v>220333.59</v>
+      </c>
+      <c r="BM19" s="1" t="n">
+        <v>915786.53</v>
+      </c>
+      <c r="BN19" s="1" t="n">
+        <v>220221.51</v>
+      </c>
+      <c r="BO19" s="1" t="n">
+        <v>9408.209999999999</v>
+      </c>
+      <c r="BP19" s="1" t="n">
+        <v>4868003.28</v>
+      </c>
+      <c r="BQ19" s="1" t="n">
+        <v>351028.79</v>
+      </c>
+      <c r="BS19" s="1" t="n">
+        <v>218011.3</v>
+      </c>
+      <c r="BT19" s="1" t="n">
+        <v>314481.39</v>
+      </c>
+      <c r="BU19" s="1" t="n">
+        <v>888120.36</v>
+      </c>
+      <c r="BV19" s="1" t="n">
+        <v>797688.35</v>
+      </c>
+      <c r="BW19" s="1" t="n">
+        <v>30269.55</v>
+      </c>
+      <c r="BX19" s="1" t="n">
+        <v>16832.11</v>
+      </c>
+      <c r="BY19" s="1" t="n">
+        <v>55597.99</v>
+      </c>
+      <c r="BZ19" s="1" t="n">
+        <v>616845.45</v>
+      </c>
+      <c r="CA19" s="1" t="n">
+        <v>1017074.97</v>
+      </c>
+      <c r="CB19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC19" s="1" t="n">
+        <v>35729.79</v>
+      </c>
+      <c r="CD19" s="1" t="n">
+        <v>917733.22</v>
+      </c>
+      <c r="CE19" s="1" t="n">
+        <v>11235.74</v>
+      </c>
+      <c r="CF19" s="1" t="n">
+        <v>45593.79</v>
+      </c>
+      <c r="CG19" s="1" t="n">
+        <v>407793.74</v>
+      </c>
+      <c r="CH19" s="1" t="n">
+        <v>37222.06</v>
+      </c>
+      <c r="CI19" s="1" t="n">
+        <v>2215892.21</v>
+      </c>
+      <c r="CJ19" s="1" t="n">
+        <v>749039.92</v>
+      </c>
+      <c r="CK19" s="1" t="n">
+        <v>3071.7</v>
+      </c>
+      <c r="CL19" s="1" t="n">
+        <v>250115.36</v>
+      </c>
+      <c r="CM19" s="1" t="n">
+        <v>14184.29</v>
+      </c>
+      <c r="CN19" s="1" t="n">
+        <v>16916.83</v>
+      </c>
+      <c r="CO19" s="1" t="n">
+        <v>60913.21</v>
+      </c>
+      <c r="CP19" s="1" t="n">
+        <v>255255.64</v>
+      </c>
+      <c r="CQ19" s="1" t="n">
+        <v>38761.65</v>
+      </c>
+      <c r="CR19" s="1" t="n">
+        <v>548.22</v>
+      </c>
+      <c r="CS19" s="1" t="n">
+        <v>143148.05</v>
+      </c>
+      <c r="CT19" s="1" t="n">
+        <v>16358.86</v>
+      </c>
+      <c r="CV19" s="1" t="n">
+        <v>549648.7</v>
+      </c>
+      <c r="CW19" s="1" t="n">
+        <v>351048.4</v>
+      </c>
+      <c r="CX19" s="1" t="n">
+        <v>4294.61</v>
+      </c>
+      <c r="CY19" s="1" t="n">
+        <v>1376553.69</v>
+      </c>
+      <c r="CZ19" s="1" t="n">
+        <v>29863.95</v>
+      </c>
+      <c r="DA19" s="1" t="n">
+        <v>84104.58</v>
+      </c>
+      <c r="DB19" s="1" t="n">
+        <v>33224.67</v>
+      </c>
+      <c r="DC19" s="1" t="n">
+        <v>18235.01</v>
+      </c>
+      <c r="DD19" s="1" t="n">
+        <v>11012.93</v>
+      </c>
+      <c r="DE19" s="1" t="n">
+        <v>30145.87</v>
+      </c>
+      <c r="DG19" s="1" t="n">
+        <v>32235.36</v>
+      </c>
+      <c r="DH19" s="1" t="n">
+        <v>54211.21</v>
+      </c>
+      <c r="DI19" s="1" t="n">
+        <v>39167.23</v>
+      </c>
+      <c r="DJ19" s="1" t="n">
+        <v>47299.14</v>
+      </c>
+      <c r="DK19" s="1" t="n">
+        <v>127780.97</v>
+      </c>
+      <c r="DL19" s="1" t="n">
+        <v>1947.57</v>
+      </c>
+      <c r="DM19" s="1" t="n">
+        <v>73282.55</v>
+      </c>
+      <c r="DN19" s="1" t="n">
+        <v>74412.5</v>
+      </c>
+      <c r="DO19" s="1" t="n">
+        <v>209813.85</v>
+      </c>
+      <c r="DP19" s="1" t="n">
+        <v>1354.71</v>
+      </c>
+      <c r="DQ19" s="1" t="n">
+        <v>41459.31</v>
+      </c>
+      <c r="DR19" s="1" t="n">
+        <v>79041.25</v>
+      </c>
+      <c r="DS19" s="1" t="n">
+        <v>125444.55</v>
+      </c>
+      <c r="DT19" s="1" t="n">
+        <v>6496.07</v>
+      </c>
+      <c r="DV19" s="1" t="n">
+        <v>3962961</v>
+      </c>
+      <c r="DW19" s="1" t="n">
+        <v>299.25</v>
+      </c>
+      <c r="DX19" s="1" t="n">
+        <v>158898.24</v>
+      </c>
+      <c r="DY19" s="1" t="n">
+        <v>2488.61</v>
+      </c>
+      <c r="DZ19" s="1" t="n">
+        <v>55698.28</v>
+      </c>
+      <c r="EA19" s="1" t="n">
+        <v>16062.85</v>
+      </c>
+      <c r="EB19" s="1" t="n">
+        <v>5217.48</v>
+      </c>
+      <c r="EC19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="ED19" s="1" t="n">
+        <v>956277.35</v>
+      </c>
+      <c r="EE19" s="1" t="n">
+        <v>8965.360000000001</v>
+      </c>
+      <c r="EF19" s="1" t="n">
+        <v>944.88</v>
+      </c>
+      <c r="EG19" s="1" t="n">
+        <v>160833.51</v>
+      </c>
+      <c r="EH19" s="1" t="n">
+        <v>3103.82</v>
+      </c>
+      <c r="EI19" s="1" t="n">
+        <v>211295.39</v>
+      </c>
+      <c r="EJ19" s="1" t="n">
+        <v>4040.01</v>
+      </c>
+      <c r="EK19" s="1" t="n">
+        <v>29669.27</v>
+      </c>
+      <c r="EL19" s="1" t="n">
+        <v>492.25</v>
+      </c>
+      <c r="EM19" s="1" t="n">
+        <v>802.38</v>
+      </c>
+      <c r="EN19" s="1" t="n">
+        <v>10164.13</v>
+      </c>
+      <c r="EO19" s="1" t="n">
+        <v>51202.79</v>
+      </c>
+      <c r="EP19" s="1" t="n">
+        <v>2609985.51</v>
+      </c>
+      <c r="EQ19" s="1" t="n">
+        <v>24.85</v>
+      </c>
+      <c r="ER19" s="1" t="n">
+        <v>1164.03</v>
+      </c>
+      <c r="ES19" s="1" t="n">
+        <v>2407.96</v>
+      </c>
+      <c r="ET19" s="1" t="n">
+        <v>54.49</v>
+      </c>
+      <c r="EU19" s="1" t="n">
+        <v>27087.7</v>
+      </c>
+      <c r="EV19" s="1" t="n">
+        <v>55481.5</v>
+      </c>
+      <c r="EX19" s="1" t="n">
+        <v>296703.64</v>
+      </c>
+      <c r="EY19" s="1" t="n">
+        <v>4918.96</v>
+      </c>
+      <c r="EZ19" s="1" t="n">
+        <v>5561.18</v>
+      </c>
+      <c r="FB19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="FC19" s="1" t="n">
+        <v>75803.16</v>
+      </c>
+      <c r="FD19" s="1" t="n">
+        <v>9485.84</v>
+      </c>
+      <c r="FE19" s="1" t="n">
+        <v>224755.02</v>
+      </c>
+      <c r="FF19" s="1" t="n">
+        <v>349.33</v>
+      </c>
+      <c r="FG19" s="1" t="n">
+        <v>7913.05</v>
+      </c>
+      <c r="FH19" s="1" t="n">
+        <v>33143.6</v>
+      </c>
+      <c r="FI19" s="1" t="n">
+        <v>6401.43</v>
+      </c>
+      <c r="FK19" s="1" t="n">
+        <v>8567.940000000001</v>
+      </c>
+      <c r="FL19" s="1" t="n">
+        <v>6714.25</v>
+      </c>
+      <c r="FM19" s="1" t="n">
+        <v>15631.23</v>
+      </c>
+      <c r="FN19" s="1" t="n">
+        <v>177394.26</v>
+      </c>
+      <c r="FO19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="FP19" s="1" t="n">
+        <v>282.44</v>
+      </c>
+      <c r="FQ19" s="1" t="n">
+        <v>35340.24</v>
+      </c>
+      <c r="FR19" s="1" t="n">
+        <v>236797.72</v>
+      </c>
+      <c r="FS19" s="1" t="n">
+        <v>979578.4</v>
+      </c>
+      <c r="FT19" s="1" t="n">
+        <v>40081.56</v>
+      </c>
+      <c r="FU19" s="1" t="n">
+        <v>9292.290000000001</v>
+      </c>
+      <c r="FV19" s="1" t="n">
+        <v>63769.73</v>
+      </c>
+      <c r="FW19" s="1" t="n">
+        <v>505.77</v>
+      </c>
+      <c r="FX19" s="1" t="n">
+        <v>3300.07</v>
+      </c>
+      <c r="FY19" s="1" t="n">
+        <v>1276425.75</v>
+      </c>
+      <c r="FZ19" s="1" t="n">
+        <v>42867.44</v>
+      </c>
+      <c r="GA19" s="1" t="n">
+        <v>40203.94</v>
+      </c>
+      <c r="GB19" s="1" t="n">
+        <v>3516.45</v>
+      </c>
+      <c r="GC19" s="1" t="n">
+        <v>558215.63</v>
+      </c>
+      <c r="GD19" s="1" t="n">
+        <v>406.92</v>
+      </c>
+      <c r="GE19" s="1" t="n">
+        <v>166582.05</v>
+      </c>
+      <c r="GF19" s="1" t="n">
+        <v>3202.63</v>
+      </c>
+      <c r="GG19" s="1" t="n">
+        <v>218.31</v>
+      </c>
+      <c r="GH19" s="1" t="n">
+        <v>23354.26</v>
+      </c>
+      <c r="GI19" s="1" t="n">
+        <v>98643.16</v>
+      </c>
+      <c r="GJ19" s="1" t="n">
+        <v>7276.34</v>
+      </c>
+      <c r="GK19" s="1" t="n">
+        <v>65875.32000000001</v>
+      </c>
+      <c r="GL19" s="1" t="n">
+        <v>274.46</v>
+      </c>
+      <c r="GM19" s="1" t="n">
+        <v>5405835.47</v>
+      </c>
+      <c r="GN19" s="1" t="n">
+        <v>122.98</v>
+      </c>
+      <c r="GO19" s="1" t="n">
+        <v>68120.11</v>
+      </c>
+      <c r="GP19" s="1" t="n">
+        <v>20416.06</v>
+      </c>
+      <c r="GQ19" s="1" t="n">
+        <v>57283.52</v>
+      </c>
+      <c r="GR19" s="1" t="n">
+        <v>180421.68</v>
+      </c>
+      <c r="GS19" s="1" t="n">
+        <v>3214.68</v>
+      </c>
+      <c r="GT19" s="1" t="n">
+        <v>375501.9</v>
+      </c>
+      <c r="GU19" s="1" t="n">
+        <v>134.76</v>
+      </c>
+      <c r="GV19" s="1" t="n">
+        <v>44813.41</v>
+      </c>
+      <c r="GX19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="GY19" s="1" t="n">
+        <v>167166.43</v>
+      </c>
+      <c r="GZ19" s="1" t="n">
+        <v>997.5</v>
+      </c>
+      <c r="HA19" s="1" t="n">
+        <v>2667.67</v>
+      </c>
+      <c r="HB19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="HC19" s="1" t="n">
+        <v>3174.83</v>
+      </c>
+      <c r="HD19" s="1" t="n">
+        <v>952.37</v>
+      </c>
+      <c r="HE19" s="1" t="n">
+        <v>4630.24</v>
+      </c>
+      <c r="HF19" s="1" t="n">
+        <v>26574.37</v>
+      </c>
+      <c r="HG19" s="1" t="n">
+        <v>63.93</v>
+      </c>
+      <c r="HH19" s="1" t="n">
+        <v>80790.22</v>
+      </c>
+      <c r="HI19" s="1" t="n">
+        <v>10707.16</v>
+      </c>
+      <c r="HJ19" s="1" t="n">
+        <v>32889.29</v>
+      </c>
+      <c r="HK19" s="1" t="n">
+        <v>48235.71</v>
+      </c>
+      <c r="HL19" s="1" t="n">
+        <v>23845.87</v>
+      </c>
+      <c r="HM19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="HN19" s="1" t="n">
+        <v>41790.92</v>
+      </c>
+      <c r="HO19" s="1" t="n">
+        <v>8303.780000000001</v>
+      </c>
+      <c r="HP19" s="1" t="n">
+        <v>90472.58</v>
+      </c>
+      <c r="HQ19" s="1" t="n">
+        <v>34550.53</v>
+      </c>
+      <c r="HR19" s="1" t="n">
+        <v>11675.37</v>
+      </c>
+      <c r="HS19" s="1" t="n">
+        <v>4607.44</v>
+      </c>
+      <c r="HT19" s="1" t="n">
+        <v>18333.27</v>
+      </c>
+      <c r="HU19" s="1" t="n">
+        <v>21874.25</v>
+      </c>
+      <c r="HV19" s="1" t="n">
+        <v>7160.34</v>
+      </c>
+      <c r="HW19" s="1" t="n">
+        <v>5805.47</v>
+      </c>
+      <c r="HX19" s="1" t="n">
+        <v>4987.52</v>
+      </c>
+      <c r="HY19" s="1" t="n">
+        <v>5766936.57</v>
+      </c>
+      <c r="HZ19" s="1" t="n">
+        <v>156508.64</v>
+      </c>
+      <c r="IA19" s="1" t="n">
+        <v>45877.34</v>
+      </c>
+      <c r="IB19" s="1" t="n">
+        <v>24466.64</v>
+      </c>
+      <c r="IC19" s="1" t="n">
+        <v>113291.74</v>
+      </c>
+      <c r="ID19" s="1" t="n">
+        <v>1842.1</v>
+      </c>
+      <c r="IE19" s="1" t="n">
+        <v>22340.57</v>
+      </c>
+      <c r="IF19" s="1" t="n">
+        <v>30258.47</v>
+      </c>
+      <c r="IG19" s="1" t="n">
+        <v>17462.86</v>
+      </c>
+      <c r="IH19" s="1" t="n">
+        <v>73892.69</v>
+      </c>
+      <c r="II19" s="1" t="n">
+        <v>56357.37</v>
+      </c>
+      <c r="IJ19" s="1" t="n">
+        <v>308042.83</v>
+      </c>
+      <c r="IK19" s="1" t="n">
+        <v>409055.35</v>
+      </c>
+      <c r="IL19" s="1" t="n">
+        <v>93182.27</v>
+      </c>
+      <c r="IM19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="IN19" s="1" t="n">
+        <v>28.59</v>
+      </c>
+      <c r="IO19" s="1" t="n">
+        <v>2938</v>
+      </c>
+      <c r="IP19" s="1" t="n">
+        <v>45363.93</v>
+      </c>
+      <c r="IQ19" s="1" t="n">
+        <v>120.05</v>
+      </c>
+      <c r="IR19" s="1" t="n">
+        <v>206.65</v>
+      </c>
+      <c r="IS19" s="1" t="n">
+        <v>605.8099999999999</v>
+      </c>
+      <c r="IT19" s="1" t="n">
+        <v>12898.66</v>
+      </c>
+      <c r="IU19" s="1" t="n">
+        <v>4048.51</v>
+      </c>
+      <c r="IV19" s="1" t="n">
+        <v>28432.11</v>
+      </c>
+      <c r="IW19" s="1" t="n">
+        <v>10924.68</v>
+      </c>
+      <c r="IX19" s="1" t="n">
+        <v>134857.16</v>
+      </c>
+      <c r="IY19" s="1" t="n">
+        <v>32718.84</v>
+      </c>
+      <c r="IZ19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="JA19" s="1" t="n">
+        <v>641.92</v>
+      </c>
+      <c r="JB19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="JC19" s="1" t="n">
+        <v>392399.36</v>
+      </c>
+      <c r="JD19" s="1" t="n">
+        <v>25483.33</v>
+      </c>
+      <c r="JE19" s="1" t="n">
+        <v>405.08</v>
+      </c>
+      <c r="JF19" s="1" t="n">
+        <v>3298.89</v>
+      </c>
+      <c r="JG19" s="1" t="n">
+        <v>216038.32</v>
+      </c>
+      <c r="JH19" s="1" t="n">
+        <v>61037.46</v>
+      </c>
+      <c r="JI19" s="1" t="n">
+        <v>1785.61</v>
+      </c>
+      <c r="JJ19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="JK19" s="1" t="n">
+        <v>21918.46</v>
+      </c>
+      <c r="JM19" s="1" t="n">
+        <v>2746.92</v>
+      </c>
+      <c r="JN19" s="1" t="n">
+        <v>5602.4</v>
+      </c>
+      <c r="JO19" s="1" t="n">
+        <v>62577.61</v>
+      </c>
+      <c r="JP19" s="1" t="n">
+        <v>888.91</v>
+      </c>
+      <c r="JQ19" s="1" t="n">
+        <v>2877.92</v>
+      </c>
+      <c r="JR19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="JS19" s="1" t="n">
+        <v>57.87</v>
+      </c>
+      <c r="JT19" s="1" t="n">
+        <v>593.53</v>
+      </c>
+      <c r="JU19" s="1" t="n">
+        <v>83262.42999999999</v>
+      </c>
+      <c r="JV19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="JX19" s="1" t="n">
+        <v>496.2</v>
+      </c>
+      <c r="JY19" s="1" t="n">
+        <v>15008.6</v>
+      </c>
+      <c r="JZ19" s="1" t="n">
+        <v>7789658.57</v>
+      </c>
+      <c r="KA19" s="1" t="n">
+        <v>1122.5</v>
+      </c>
+      <c r="KB19" s="1" t="n">
+        <v>8927.129999999999</v>
+      </c>
+      <c r="KC19" s="1" t="n">
+        <v>32085.36</v>
+      </c>
+      <c r="KD19" s="1" t="n">
+        <v>797.9</v>
+      </c>
+      <c r="KE19" s="1" t="n">
+        <v>1952.08</v>
+      </c>
+      <c r="KF19" s="1" t="n">
+        <v>6092.83</v>
+      </c>
+      <c r="KG19" s="1" t="n">
+        <v>8572.139999999999</v>
+      </c>
+      <c r="KH19" s="1" t="n">
+        <v>1933.56</v>
+      </c>
+      <c r="KI19" s="1" t="n">
+        <v>6872.5</v>
+      </c>
+      <c r="KJ19" s="1" t="n">
+        <v>92676.36</v>
+      </c>
+      <c r="KK19" s="1" t="n">
+        <v>215.59</v>
+      </c>
+      <c r="KM19" s="1" t="n">
+        <v>75.14</v>
+      </c>
+      <c r="KN19" s="1" t="n">
+        <v>19046.13</v>
+      </c>
+      <c r="KO19" s="1" t="n">
+        <v>31133.54</v>
+      </c>
+      <c r="KP19" s="1" t="n">
+        <v>39900.24</v>
+      </c>
+      <c r="KQ19" s="1" t="n">
+        <v>518.54</v>
+      </c>
+      <c r="KR19" s="1" t="n">
+        <v>14406.3</v>
+      </c>
+      <c r="KS19" s="1" t="n">
+        <v>16949.51</v>
+      </c>
+      <c r="KT19" s="1" t="n">
+        <v>1006.27</v>
+      </c>
+      <c r="KU19" s="1" t="n">
+        <v>1548.35</v>
+      </c>
+      <c r="KV19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="KW19" s="1" t="n">
+        <v>25759.79</v>
+      </c>
+      <c r="KX19" s="1" t="n">
+        <v>11676.92</v>
+      </c>
+      <c r="KY19" s="1" t="n">
+        <v>4944.83</v>
+      </c>
+      <c r="KZ19" s="1" t="n">
+        <v>37.39</v>
+      </c>
+      <c r="LA19" s="1" t="n">
+        <v>14185.52</v>
+      </c>
+      <c r="LB19" s="1" t="n">
+        <v>12246.75</v>
+      </c>
+      <c r="LC19" s="1" t="n">
+        <v>1153.06</v>
+      </c>
+      <c r="LD19" s="1" t="n">
+        <v>166180.66</v>
+      </c>
+      <c r="LE19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="LF19" s="1" t="n">
+        <v>1249.91</v>
+      </c>
+      <c r="LG19" s="1" t="n">
+        <v>713.66</v>
+      </c>
+      <c r="LI19" s="1" t="n">
+        <v>15434.32</v>
+      </c>
+      <c r="LJ19" s="1" t="n">
+        <v>5712.95</v>
+      </c>
+      <c r="LK19" s="1" t="n">
+        <v>6038.04</v>
+      </c>
+      <c r="LL19" s="1" t="n">
+        <v>594.77</v>
+      </c>
+      <c r="LO19" s="1" t="n">
+        <v>1995</v>
+      </c>
+      <c r="LP19" s="1" t="n">
+        <v>1523.67</v>
+      </c>
+      <c r="LQ19" s="1" t="n">
+        <v>1061.61</v>
+      </c>
+      <c r="LR19" s="1" t="n">
+        <v>1359.36</v>
+      </c>
+      <c r="LS19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="LT19" s="1" t="n">
+        <v>7853.8</v>
+      </c>
+      <c r="LU19" s="1" t="n">
+        <v>401.31</v>
+      </c>
+      <c r="LV19" s="1" t="n">
+        <v>13046.69</v>
+      </c>
+      <c r="LW19" s="1" t="n">
+        <v>315.95</v>
+      </c>
+      <c r="LX19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="LY19" s="1" t="n">
+        <v>30.08</v>
+      </c>
+      <c r="LZ19" s="1" t="n">
+        <v>548.61</v>
+      </c>
+      <c r="MA19" s="1" t="n">
+        <v>2378.76</v>
+      </c>
+      <c r="MB19" s="1" t="n">
+        <v>373.53</v>
+      </c>
+      <c r="MC19" s="1" t="n">
+        <v>63202.42</v>
+      </c>
+      <c r="MD19" s="1" t="n">
+        <v>7776.47</v>
+      </c>
+      <c r="ME19" s="1" t="n">
+        <v>16.7</v>
+      </c>
+      <c r="MF19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="MG19" s="1" t="n">
+        <v>2535.04</v>
+      </c>
+      <c r="MH19" s="1" t="n">
+        <v>68.25</v>
+      </c>
+      <c r="MI19" s="1" t="n">
+        <v>35409.81</v>
+      </c>
+      <c r="MJ19" s="1" t="n">
+        <v>2812.54</v>
+      </c>
+      <c r="MK19" s="1" t="n">
+        <v>2083.31</v>
+      </c>
+      <c r="ML19" s="1" t="n">
+        <v>32.77</v>
+      </c>
+      <c r="MM19" s="1" t="n">
+        <v>4504.16</v>
+      </c>
+      <c r="MN19" s="1" t="n">
+        <v>1189.38</v>
+      </c>
+      <c r="MO19" s="1" t="n">
+        <v>43102.1</v>
+      </c>
+      <c r="MP19" s="1" t="n">
+        <v>14003.8</v>
+      </c>
+      <c r="MQ19" s="1" t="n">
+        <v>792.98</v>
+      </c>
+      <c r="MR19" s="1" t="n">
+        <v>7985.73</v>
+      </c>
+      <c r="MS19" s="1" t="n">
+        <v>1048.31</v>
+      </c>
+      <c r="MT19" s="1" t="n">
+        <v>5652.66</v>
+      </c>
+      <c r="MU19" s="1" t="n">
+        <v>8821.139999999999</v>
+      </c>
+      <c r="MV19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="MW19" s="1" t="n">
+        <v>4815.43</v>
+      </c>
+      <c r="MX19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="MY19" s="1" t="n">
+        <v>1132.42</v>
+      </c>
+      <c r="MZ19" s="1" t="n">
+        <v>18227.92</v>
+      </c>
+      <c r="NA19" s="1" t="n">
+        <v>77.05</v>
+      </c>
+      <c r="NB19" s="1" t="n">
+        <v>286.1</v>
+      </c>
+      <c r="NC19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="ND19" s="1" t="n">
+        <v>1145</v>
+      </c>
+      <c r="NE19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="NF19" s="1" t="n">
+        <v>815.16</v>
+      </c>
+      <c r="NG19" s="1" t="n">
+        <v>53.2</v>
+      </c>
+      <c r="NH19" s="1" t="n">
+        <v>2816094.97</v>
+      </c>
+      <c r="PB19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="PK19" s="1" t="n">
+        <v>2391.46</v>
+      </c>
+      <c r="PV19" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -22746,7 +23823,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BXW18"/>
+  <dimension ref="A1:BXW19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23504,6 +24581,48 @@
       </c>
       <c r="M18" s="1" t="n">
         <v>228841.241468</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>13</v>
+      </c>
+      <c r="B19" s="1" t="n">
+        <v>228487736.4</v>
+      </c>
+      <c r="C19" s="1" t="n">
+        <v>53781951.59154</v>
+      </c>
+      <c r="D19" s="1">
+        <f>AVERAGE(C13:C19)</f>
+        <v/>
+      </c>
+      <c r="E19" s="1" t="n">
+        <v>728928.2594</v>
+      </c>
+      <c r="F19" s="1" t="n">
+        <v>1553285.7466</v>
+      </c>
+      <c r="G19" s="1" t="n">
+        <v>469876.1892</v>
+      </c>
+      <c r="H19" s="1" t="n">
+        <v>234625.6547</v>
+      </c>
+      <c r="I19" s="1" t="n">
+        <v>1837211.5926</v>
+      </c>
+      <c r="J19" s="1" t="n">
+        <v>68353.90429999999</v>
+      </c>
+      <c r="K19" s="1" t="n">
+        <v>4783.8508</v>
+      </c>
+      <c r="L19" s="1" t="n">
+        <v>4051.9972</v>
+      </c>
+      <c r="M19" s="1" t="n">
+        <v>40389.522186</v>
       </c>
     </row>
   </sheetData>
@@ -23517,7 +24636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BXW18"/>
+  <dimension ref="A1:BXW19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29482,6 +30601,327 @@
         <v>0</v>
       </c>
       <c r="DB18" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>13</v>
+      </c>
+      <c r="B19" s="1" t="n">
+        <v>326404.9117164645</v>
+      </c>
+      <c r="C19" s="1" t="n">
+        <v>159808.6975110888</v>
+      </c>
+      <c r="D19" s="1">
+        <f>AVERAGE(C13:C19)</f>
+        <v/>
+      </c>
+      <c r="E19" s="1" t="n">
+        <v>3754624.229601813</v>
+      </c>
+      <c r="F19" s="1" t="n">
+        <v>7906.5488364685</v>
+      </c>
+      <c r="G19" s="1" t="n">
+        <v>210650.4004093856</v>
+      </c>
+      <c r="H19" s="1" t="n">
+        <v>92454.4904311326</v>
+      </c>
+      <c r="I19" s="1" t="n">
+        <v>14048.75735484302</v>
+      </c>
+      <c r="J19" s="1" t="n">
+        <v>742.628</v>
+      </c>
+      <c r="K19" s="1" t="n">
+        <v>1621.600168404</v>
+      </c>
+      <c r="L19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" s="1" t="n">
+        <v>997.3321343568</v>
+      </c>
+      <c r="N19" s="1" t="n">
+        <v>3753.29762</v>
+      </c>
+      <c r="O19" s="1" t="n">
+        <v>997.3200000000001</v>
+      </c>
+      <c r="P19" s="1" t="n">
+        <v>540.00548532</v>
+      </c>
+      <c r="Q19" s="1" t="n">
+        <v>360.1366343232</v>
+      </c>
+      <c r="R19" s="1" t="n">
+        <v>350.0626839638</v>
+      </c>
+      <c r="S19" s="1" t="n">
+        <v>1292.3321362964</v>
+      </c>
+      <c r="T19" s="1" t="n">
+        <v>1262.0371</v>
+      </c>
+      <c r="U19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="V19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="W19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="X19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI19" s="1" t="n">
+        <v>846.1776</v>
+      </c>
+      <c r="BJ19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BS19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BV19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BY19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE19" s="1" t="n">
+        <v>2954.6642688</v>
+      </c>
+      <c r="CF19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CG19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CH19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CJ19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CK19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CM19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CN19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO19" s="1" t="n">
+        <v>48.6486</v>
+      </c>
+      <c r="CP19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CQ19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CS19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CT19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CU19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CV19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CW19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CX19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CY19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="DA19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="DB19" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -29496,7 +30936,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BXW18"/>
+  <dimension ref="A1:BXW19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31599,6 +33039,126 @@
       </c>
       <c r="AM18" s="1" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>13</v>
+      </c>
+      <c r="B19" s="1" t="n">
+        <v>1608892.46</v>
+      </c>
+      <c r="C19" s="1">
+        <f>AVERAGE(B13:B19)</f>
+        <v/>
+      </c>
+      <c r="D19" s="1" t="n">
+        <v>86464.98</v>
+      </c>
+      <c r="E19" s="1" t="n">
+        <v>263159.39</v>
+      </c>
+      <c r="F19" s="1" t="n">
+        <v>76577.84</v>
+      </c>
+      <c r="G19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="1" t="n">
+        <v>94999.88</v>
+      </c>
+      <c r="I19" s="1" t="n">
+        <v>65623.03999999999</v>
+      </c>
+      <c r="J19" s="1" t="n">
+        <v>69435.91</v>
+      </c>
+      <c r="K19" s="1" t="n">
+        <v>6943.14</v>
+      </c>
+      <c r="L19" s="1" t="n">
+        <v>58290.37</v>
+      </c>
+      <c r="M19" s="1" t="n">
+        <v>46651.04</v>
+      </c>
+      <c r="N19" s="1" t="n">
+        <v>519.62</v>
+      </c>
+      <c r="O19" s="1" t="n">
+        <v>498.95</v>
+      </c>
+      <c r="P19" s="1" t="n">
+        <v>560.14</v>
+      </c>
+      <c r="Q19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="R19" s="1" t="n">
+        <v>81824.55</v>
+      </c>
+      <c r="S19" s="1" t="n">
+        <v>9364.82</v>
+      </c>
+      <c r="T19" s="1" t="n">
+        <v>15162.59</v>
+      </c>
+      <c r="U19" s="1" t="n">
+        <v>109182.29</v>
+      </c>
+      <c r="V19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="W19" s="1" t="n">
+        <v>247852.44</v>
+      </c>
+      <c r="X19" s="1" t="n">
+        <v>4946</v>
+      </c>
+      <c r="Y19" s="1" t="n">
+        <v>508.23</v>
+      </c>
+      <c r="Z19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA19" s="1" t="n">
+        <v>1003.05</v>
+      </c>
+      <c r="AB19" s="1" t="n">
+        <v>1761.17</v>
+      </c>
+      <c r="AC19" s="1" t="n">
+        <v>2219.54</v>
+      </c>
+      <c r="AD19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE19" s="1" t="n">
+        <v>515.42</v>
+      </c>
+      <c r="AF19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH19" s="1" t="n">
+        <v>100617.36</v>
+      </c>
+      <c r="AI19" s="1" t="n">
+        <v>2691.95</v>
+      </c>
+      <c r="AJ19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK19" s="1" t="n">
+        <v>606523.67</v>
+      </c>
+      <c r="AL19" s="1" t="n">
+        <v>1858.25</v>
+      </c>
+      <c r="AM19" s="1" t="n">
+        <v>500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>